<commit_message>
Final fit (I hope) with least square.
</commit_message>
<xml_diff>
--- a/Files/data gabriel/field_dep_5_7_GHz_0deg.xlsx
+++ b/Files/data gabriel/field_dep_5_7_GHz_0deg.xlsx
@@ -1,14 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Python\continuum-Doppler-shift\Files\data gabriel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D77D84D-7279-4F58-8440-552B7E051BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -54,11 +61,16 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -81,21 +93,351 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:M75"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="30.85546875" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -133,30 +475,30 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2">
-        <v>6.3224705589605897e-05</v>
+        <v>6.3224705589605897E-5</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>3.1346220052325097e-05</v>
+        <v>3.1346220052325097E-5</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>6.2993773993993502e-05</v>
+        <v>6.2993773993993502E-5</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>2.8966275322346902e-05</v>
+        <v>2.8966275322346902E-5</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -171,68 +513,68 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3">
-        <v>-0.000117868335889597</v>
+        <v>-1.17868335889597E-4</v>
       </c>
       <c r="C3">
-        <v>6.2099615724817801e-05</v>
+        <v>6.2099615724817801E-5</v>
       </c>
       <c r="D3">
-        <v>-6.5394768914332302e-05</v>
+        <v>-6.5394768914332302E-5</v>
       </c>
       <c r="E3">
-        <v>2.9054001044463202e-05</v>
+        <v>2.9054001044463202E-5</v>
       </c>
       <c r="F3">
-        <v>-5.9045710571679602e-05</v>
+        <v>-5.9045710571679602E-5</v>
       </c>
       <c r="G3">
-        <v>6.3228500947020097e-05</v>
+        <v>6.3228500947020097E-5</v>
       </c>
       <c r="H3">
-        <v>8.7369792541050199e-05</v>
+        <v>8.7369792541050199E-5</v>
       </c>
       <c r="I3">
-        <v>2.68029744727775e-05</v>
+        <v>2.68029744727775E-5</v>
       </c>
       <c r="J3">
-        <v>0.0050000000000000001</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="K3">
-        <v>0.0050000000000000001</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="L3">
-        <v>0.0050000000000000001</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="M3">
-        <v>0.0050000000000000001</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4">
-        <v>-4.2593670489565999e-05</v>
+        <v>-4.2593670489565999E-5</v>
       </c>
       <c r="C4">
-        <v>5.7988491007806301e-05</v>
+        <v>5.7988491007806301E-5</v>
       </c>
       <c r="D4">
-        <v>-7.7776098909075407e-06</v>
+        <v>-7.7776098909075407E-6</v>
       </c>
       <c r="E4">
-        <v>2.62960002323122e-05</v>
+        <v>2.62960002323122E-5</v>
       </c>
       <c r="F4">
-        <v>-0.00017283976299566699</v>
+        <v>-1.7283976299566699E-4</v>
       </c>
       <c r="G4">
-        <v>6.37824568314808e-05</v>
+        <v>6.37824568314808E-5</v>
       </c>
       <c r="H4">
-        <v>1.9374836945641701e-06</v>
+        <v>1.9374836945641701E-6</v>
       </c>
       <c r="I4">
-        <v>2.6762720776148499e-05</v>
+        <v>2.6762720776148499E-5</v>
       </c>
       <c r="J4">
         <v>0.01</v>
@@ -247,68 +589,68 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5">
-        <v>9.6219896350138801e-05</v>
+        <v>9.6219896350138801E-5</v>
       </c>
       <c r="C5">
-        <v>6.2613397122517506e-05</v>
+        <v>6.2613397122517506E-5</v>
       </c>
       <c r="D5">
-        <v>-0.000154342232753327</v>
+        <v>-1.54342232753327E-4</v>
       </c>
       <c r="E5">
-        <v>2.5325436717126901e-05</v>
+        <v>2.5325436717126901E-5</v>
       </c>
       <c r="F5">
-        <v>-0.00034243214347857499</v>
+        <v>-3.4243214347857499E-4</v>
       </c>
       <c r="G5">
-        <v>5.4297846297996599e-05</v>
+        <v>5.4297846297996599E-5</v>
       </c>
       <c r="H5">
-        <v>-3.8203296426855901e-05</v>
+        <v>-3.8203296426855901E-5</v>
       </c>
       <c r="I5">
-        <v>2.6587559159979699e-05</v>
+        <v>2.6587559159979699E-5</v>
       </c>
       <c r="J5">
-        <v>0.014999999999999999</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="K5">
-        <v>0.014999999999999999</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="L5">
-        <v>0.014999999999999999</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="M5">
-        <v>0.014999999999999999</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6">
-        <v>-5.0576410659033801e-05</v>
+        <v>-5.0576410659033801E-5</v>
       </c>
       <c r="C6">
-        <v>6.3293075814739407e-05</v>
+        <v>6.3293075814739407E-5</v>
       </c>
       <c r="D6">
-        <v>-0.00025240343859617398</v>
+        <v>-2.5240343859617398E-4</v>
       </c>
       <c r="E6">
-        <v>2.6976929196349402e-05</v>
+        <v>2.6976929196349402E-5</v>
       </c>
       <c r="F6">
-        <v>-0.00053972243377828604</v>
+        <v>-5.3972243377828604E-4</v>
       </c>
       <c r="G6">
-        <v>6.2470808084243403e-05</v>
+        <v>6.2470808084243403E-5</v>
       </c>
       <c r="H6">
-        <v>-9.2385153960279696e-05</v>
+        <v>-9.2385153960279696E-5</v>
       </c>
       <c r="I6">
-        <v>2.3948500247222001e-05</v>
+        <v>2.3948500247222001E-5</v>
       </c>
       <c r="J6">
         <v>0.02</v>
@@ -323,638 +665,638 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7">
-        <v>-8.1134584385200495e-05</v>
+        <v>-8.1134584385200495E-5</v>
       </c>
       <c r="C7">
-        <v>5.9363776358236298e-05</v>
+        <v>5.9363776358236298E-5</v>
       </c>
       <c r="D7">
-        <v>-0.00047446607859092798</v>
+        <v>-4.7446607859092798E-4</v>
       </c>
       <c r="E7">
-        <v>2.6472534189005401e-05</v>
+        <v>2.6472534189005401E-5</v>
       </c>
       <c r="F7">
-        <v>-0.00087454513804661603</v>
+        <v>-8.7454513804661603E-4</v>
       </c>
       <c r="G7">
-        <v>6.0612470873883303e-05</v>
+        <v>6.0612470873883303E-5</v>
       </c>
       <c r="H7">
-        <v>-0.000403862136741194</v>
+        <v>-4.03862136741194E-4</v>
       </c>
       <c r="I7">
-        <v>2.7728571989236801e-05</v>
+        <v>2.7728571989236801E-5</v>
       </c>
       <c r="J7">
-        <v>0.025000000000000001</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="K7">
-        <v>0.025000000000000001</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="L7">
-        <v>0.025000000000000001</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="M7">
-        <v>0.025000000000000001</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8">
-        <v>-0.000170542202634008</v>
+        <v>-1.70542202634008E-4</v>
       </c>
       <c r="C8">
-        <v>5.9388670958285399e-05</v>
+        <v>5.9388670958285399E-5</v>
       </c>
       <c r="D8">
-        <v>-0.00078546180364136005</v>
+        <v>-7.8546180364136005E-4</v>
       </c>
       <c r="E8">
-        <v>2.84467118549763e-05</v>
+        <v>2.84467118549763E-5</v>
       </c>
       <c r="F8">
-        <v>-0.00137854665055051</v>
+        <v>-1.37854665055051E-3</v>
       </c>
       <c r="G8">
-        <v>5.4213529608058598e-05</v>
+        <v>5.4213529608058598E-5</v>
       </c>
       <c r="H8">
-        <v>-0.00066063876054102898</v>
+        <v>-6.6063876054102898E-4</v>
       </c>
       <c r="I8">
-        <v>2.54751146923671e-05</v>
+        <v>2.54751146923671E-5</v>
       </c>
       <c r="J8">
-        <v>0.029999999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="K8">
-        <v>0.029999999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="L8">
-        <v>0.029999999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="M8">
-        <v>0.029999999999999999</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9">
-        <v>-0.00015196799481564301</v>
+        <v>-1.5196799481564301E-4</v>
       </c>
       <c r="C9">
-        <v>6.7798689663421698e-05</v>
+        <v>6.7798689663421698E-5</v>
       </c>
       <c r="D9">
-        <v>-0.00107595362921736</v>
+        <v>-1.07595362921736E-3</v>
       </c>
       <c r="E9">
-        <v>2.98287261663911e-05</v>
+        <v>2.98287261663911E-5</v>
       </c>
       <c r="F9">
-        <v>-0.0020456103667876699</v>
+        <v>-2.0456103667876699E-3</v>
       </c>
       <c r="G9">
-        <v>4.9213978340314399e-05</v>
+        <v>4.9213978340314399E-5</v>
       </c>
       <c r="H9">
-        <v>-0.0010292492231585</v>
+        <v>-1.0292492231585E-3</v>
       </c>
       <c r="I9">
-        <v>2.7925222051536702e-05</v>
+        <v>2.7925222051536702E-5</v>
       </c>
       <c r="J9">
-        <v>0.035000000000000003</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="K9">
-        <v>0.035000000000000003</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="L9">
-        <v>0.035000000000000003</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="M9">
-        <v>0.035000000000000003</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10">
-        <v>-0.00026690314892415998</v>
+        <v>-2.6690314892415998E-4</v>
       </c>
       <c r="C10">
-        <v>6.1284529310499895e-05</v>
+        <v>6.1284529310499895E-5</v>
       </c>
       <c r="D10">
-        <v>-0.00150077618180732</v>
+        <v>-1.50077618180732E-3</v>
       </c>
       <c r="E10">
-        <v>3.24098176787195e-05</v>
+        <v>3.24098176787195E-5</v>
       </c>
       <c r="F10">
-        <v>-0.0028924845022096301</v>
+        <v>-2.8924845022096301E-3</v>
       </c>
       <c r="G10">
-        <v>4.5168815683192802e-05</v>
+        <v>4.5168815683192802E-5</v>
       </c>
       <c r="H10">
-        <v>-0.00144782409628889</v>
+        <v>-1.44782409628889E-3</v>
       </c>
       <c r="I10">
-        <v>3.1645075757046997e-05</v>
+        <v>3.1645075757046997E-5</v>
       </c>
       <c r="J10">
-        <v>0.040000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="K10">
-        <v>0.040000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="L10">
-        <v>0.040000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="M10">
-        <v>0.040000000000000001</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11">
-        <v>-0.00042085652496948601</v>
+        <v>-4.2085652496948601E-4</v>
       </c>
       <c r="C11">
-        <v>6.0915012085349901e-05</v>
+        <v>6.0915012085349901E-5</v>
       </c>
       <c r="D11">
-        <v>-0.0020621701333318901</v>
+        <v>-2.0621701333318901E-3</v>
       </c>
       <c r="E11">
-        <v>4.1170314969695799e-05</v>
+        <v>4.1170314969695799E-5</v>
       </c>
       <c r="F11">
-        <v>-0.0039426619046572502</v>
+        <v>-3.9426619046572502E-3</v>
       </c>
       <c r="G11">
-        <v>6.1028797479387898e-05</v>
+        <v>6.1028797479387898E-5</v>
       </c>
       <c r="H11">
-        <v>-0.0018539894628299301</v>
+        <v>-1.8539894628299301E-3</v>
       </c>
       <c r="I11">
-        <v>4.2849623370108898e-05</v>
+        <v>4.2849623370108898E-5</v>
       </c>
       <c r="J11">
-        <v>0.044999999999999998</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="K11">
-        <v>0.044999999999999998</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="L11">
-        <v>0.044999999999999998</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="M11">
-        <v>0.044999999999999998</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>4.4999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12">
-        <v>-0.000744204864513518</v>
+        <v>-7.44204864513518E-4</v>
       </c>
       <c r="C12">
-        <v>6.0014497049113299e-05</v>
+        <v>6.0014497049113299E-5</v>
       </c>
       <c r="D12">
-        <v>-0.00265477022076</v>
+        <v>-2.65477022076E-3</v>
       </c>
       <c r="E12">
-        <v>3.5302651625172903e-05</v>
+        <v>3.5302651625172903E-5</v>
       </c>
       <c r="F12">
-        <v>-0.0051524529441853003</v>
+        <v>-5.1524529441853003E-3</v>
       </c>
       <c r="G12">
-        <v>7.6222208809001993e-05</v>
+        <v>7.6222208809001993E-5</v>
       </c>
       <c r="H12">
-        <v>-0.0026613364833767499</v>
+        <v>-2.6613364833767499E-3</v>
       </c>
       <c r="I12">
-        <v>4.8534238421648499e-05</v>
+        <v>4.8534238421648499E-5</v>
       </c>
       <c r="J12">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="K12">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="L12">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="M12">
-        <v>0.050000000000000003</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13">
-        <v>-0.00089112750240273597</v>
+        <v>-8.9112750240273597E-4</v>
       </c>
       <c r="C13">
-        <v>6.2245661334734803e-05</v>
+        <v>6.2245661334734803E-5</v>
       </c>
       <c r="D13">
-        <v>-0.0033169228342538101</v>
+        <v>-3.3169228342538101E-3</v>
       </c>
       <c r="E13">
-        <v>3.3802178069071803e-05</v>
+        <v>3.3802178069071803E-5</v>
       </c>
       <c r="F13">
-        <v>-0.0067995964602417698</v>
+        <v>-6.7995964602417698E-3</v>
       </c>
       <c r="G13">
-        <v>7.8592328540651602e-05</v>
+        <v>7.8592328540651602E-5</v>
       </c>
       <c r="H13">
-        <v>-0.00343713211655718</v>
+        <v>-3.43713211655718E-3</v>
       </c>
       <c r="I13">
-        <v>4.4441799609919398e-05</v>
+        <v>4.4441799609919398E-5</v>
       </c>
       <c r="J13">
-        <v>0.055</v>
+        <v>5.5E-2</v>
       </c>
       <c r="K13">
-        <v>0.055</v>
+        <v>5.5E-2</v>
       </c>
       <c r="L13">
-        <v>0.055</v>
+        <v>5.5E-2</v>
       </c>
       <c r="M13">
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>5.5E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14">
-        <v>-0.0010391717537534099</v>
+        <v>-1.0391717537534099E-3</v>
       </c>
       <c r="C14">
-        <v>6.0374807219120501e-05</v>
+        <v>6.0374807219120501E-5</v>
       </c>
       <c r="D14">
-        <v>-0.0040117867127471901</v>
+        <v>-4.0117867127471901E-3</v>
       </c>
       <c r="E14">
-        <v>2.9073253150132399e-05</v>
+        <v>2.9073253150132399E-5</v>
       </c>
       <c r="F14">
-        <v>-0.0084122913589593108</v>
+        <v>-8.4122913589593108E-3</v>
       </c>
       <c r="G14">
-        <v>8.5352471979763099e-05</v>
+        <v>8.5352471979763099E-5</v>
       </c>
       <c r="H14">
-        <v>-0.0041801816602289104</v>
+        <v>-4.1801816602289104E-3</v>
       </c>
       <c r="I14">
-        <v>4.1886689326452098e-05</v>
+        <v>4.1886689326452098E-5</v>
       </c>
       <c r="J14">
-        <v>0.059999999999999998</v>
+        <v>0.06</v>
       </c>
       <c r="K14">
-        <v>0.059999999999999998</v>
+        <v>0.06</v>
       </c>
       <c r="L14">
-        <v>0.059999999999999998</v>
+        <v>0.06</v>
       </c>
       <c r="M14">
-        <v>0.059999999999999998</v>
-      </c>
-    </row>
-    <row r="15">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15">
-        <v>-0.0012790241173447499</v>
+        <v>-1.2790241173447499E-3</v>
       </c>
       <c r="C15">
-        <v>5.9004295179280601e-05</v>
+        <v>5.9004295179280601E-5</v>
       </c>
       <c r="D15">
-        <v>-0.0046984407783178198</v>
+        <v>-4.6984407783178198E-3</v>
       </c>
       <c r="E15">
-        <v>2.4327476988814399e-05</v>
+        <v>2.4327476988814399E-5</v>
       </c>
       <c r="F15">
-        <v>-0.0096796954863655003</v>
+        <v>-9.6796954863655003E-3</v>
       </c>
       <c r="G15">
-        <v>8.21769621331376e-05</v>
+        <v>8.21769621331376E-5</v>
       </c>
       <c r="H15">
-        <v>-0.0049894873274292598</v>
+        <v>-4.9894873274292598E-3</v>
       </c>
       <c r="I15">
-        <v>3.0733264763584001e-05</v>
+        <v>3.0733264763584001E-5</v>
       </c>
       <c r="J15">
-        <v>0.065000000000000002</v>
+        <v>6.5000000000000002E-2</v>
       </c>
       <c r="K15">
-        <v>0.065000000000000002</v>
+        <v>6.5000000000000002E-2</v>
       </c>
       <c r="L15">
-        <v>0.065000000000000002</v>
+        <v>6.5000000000000002E-2</v>
       </c>
       <c r="M15">
-        <v>0.065000000000000002</v>
-      </c>
-    </row>
-    <row r="16">
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16">
-        <v>-0.0012666497502980701</v>
+        <v>-1.2666497502980701E-3</v>
       </c>
       <c r="C16">
-        <v>6.0277024181666e-05</v>
+        <v>6.0277024181666E-5</v>
       </c>
       <c r="D16">
-        <v>-0.0054262809215399896</v>
+        <v>-5.4262809215399896E-3</v>
       </c>
       <c r="E16">
-        <v>2.2591688052352799e-05</v>
+        <v>2.2591688052352799E-5</v>
       </c>
       <c r="F16">
-        <v>-0.00990440984225276</v>
+        <v>-9.90440984225276E-3</v>
       </c>
       <c r="G16">
-        <v>8.1636528145179597e-05</v>
+        <v>8.1636528145179597E-5</v>
       </c>
       <c r="H16">
-        <v>-0.0058600013120203099</v>
+        <v>-5.8600013120203099E-3</v>
       </c>
       <c r="I16">
-        <v>2.1677560545291701e-05</v>
+        <v>2.1677560545291701E-5</v>
       </c>
       <c r="J16">
-        <v>0.070000000000000007</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="K16">
-        <v>0.070000000000000007</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="L16">
-        <v>0.070000000000000007</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="M16">
-        <v>0.070000000000000007</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17">
-        <v>-0.0013422347606198801</v>
+        <v>-1.3422347606198801E-3</v>
       </c>
       <c r="C17">
-        <v>6.2634644300773497e-05</v>
+        <v>6.2634644300773497E-5</v>
       </c>
       <c r="D17">
-        <v>-0.0063809062956029401</v>
+        <v>-6.3809062956029401E-3</v>
       </c>
       <c r="E17">
-        <v>3.4295305708851601e-05</v>
+        <v>3.4295305708851601E-5</v>
       </c>
       <c r="F17">
-        <v>-0.0132816792868664</v>
+        <v>-1.32816792868664E-2</v>
       </c>
       <c r="G17">
-        <v>8.9834462058158805e-05</v>
+        <v>8.9834462058158805E-5</v>
       </c>
       <c r="H17">
-        <v>-0.0069827576623838501</v>
+        <v>-6.9827576623838501E-3</v>
       </c>
       <c r="I17">
-        <v>2.3710419558734599e-05</v>
+        <v>2.3710419558734599E-5</v>
       </c>
       <c r="J17">
-        <v>0.074999999999999997</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="K17">
-        <v>0.074999999999999997</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="L17">
-        <v>0.074999999999999997</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="M17">
-        <v>0.074999999999999997</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18">
-        <v>-0.0016211107604351201</v>
+        <v>-1.6211107604351201E-3</v>
       </c>
       <c r="C18">
-        <v>6.2576150050711499e-05</v>
+        <v>6.2576150050711499E-5</v>
       </c>
       <c r="D18">
-        <v>-0.0076015232510085202</v>
+        <v>-7.6015232510085202E-3</v>
       </c>
       <c r="E18">
-        <v>6.1049041769088803e-05</v>
+        <v>6.1049041769088803E-5</v>
       </c>
       <c r="F18">
-        <v>-0.013993200031406401</v>
+        <v>-1.3993200031406401E-2</v>
       </c>
       <c r="G18">
-        <v>9.1858037709842804e-05</v>
+        <v>9.1858037709842804E-5</v>
       </c>
       <c r="H18">
-        <v>-0.0086041660766537301</v>
+        <v>-8.6041660766537301E-3</v>
       </c>
       <c r="I18">
-        <v>3.7573218382345201e-05</v>
+        <v>3.7573218382345201E-5</v>
       </c>
       <c r="J18">
-        <v>0.080000000000000002</v>
+        <v>0.08</v>
       </c>
       <c r="K18">
-        <v>0.080000000000000002</v>
+        <v>0.08</v>
       </c>
       <c r="L18">
-        <v>0.080000000000000002</v>
+        <v>0.08</v>
       </c>
       <c r="M18">
-        <v>0.080000000000000002</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19">
-        <v>-0.0016362899205143401</v>
+        <v>-1.6362899205143401E-3</v>
       </c>
       <c r="C19">
-        <v>5.8686752582314901e-05</v>
+        <v>5.8686752582314901E-5</v>
       </c>
       <c r="D19">
-        <v>-0.0083588651836418604</v>
+        <v>-8.3588651836418604E-3</v>
       </c>
       <c r="E19">
-        <v>6.0523732070362402e-05</v>
+        <v>6.0523732070362402E-5</v>
       </c>
       <c r="F19">
-        <v>-0.017591388656289599</v>
+        <v>-1.7591388656289599E-2</v>
       </c>
       <c r="G19">
-        <v>9.3229422663076804e-05</v>
+        <v>9.3229422663076804E-5</v>
       </c>
       <c r="H19">
-        <v>-0.0087263052907707306</v>
+        <v>-8.7263052907707306E-3</v>
       </c>
       <c r="I19">
-        <v>3.6752869656034601e-05</v>
+        <v>3.6752869656034601E-5</v>
       </c>
       <c r="J19">
-        <v>0.085000000000000006</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="K19">
-        <v>0.085000000000000006</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="L19">
-        <v>0.085000000000000006</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="M19">
-        <v>0.085000000000000006</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20">
-        <v>-0.0018014673235066899</v>
+        <v>-1.8014673235066899E-3</v>
       </c>
       <c r="C20">
-        <v>5.3341309046016103e-05</v>
+        <v>5.3341309046016103E-5</v>
       </c>
       <c r="D20">
-        <v>-0.0089275489702148395</v>
+        <v>-8.9275489702148395E-3</v>
       </c>
       <c r="E20">
-        <v>3.7557403663839503e-05</v>
+        <v>3.7557403663839503E-5</v>
       </c>
       <c r="F20">
-        <v>-0.0185402979477979</v>
+        <v>-1.85402979477979E-2</v>
       </c>
       <c r="G20">
-        <v>9.6172357968489201e-05</v>
+        <v>9.6172357968489201E-5</v>
       </c>
       <c r="H20">
-        <v>-0.0100447447657289</v>
+        <v>-1.00447447657289E-2</v>
       </c>
       <c r="I20">
-        <v>3.8369105800327102e-05</v>
+        <v>3.8369105800327102E-5</v>
       </c>
       <c r="J20">
-        <v>0.089999999999999997</v>
+        <v>0.09</v>
       </c>
       <c r="K20">
-        <v>0.089999999999999997</v>
+        <v>0.09</v>
       </c>
       <c r="L20">
-        <v>0.089999999999999997</v>
+        <v>0.09</v>
       </c>
       <c r="M20">
-        <v>0.089999999999999997</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21">
-        <v>-0.00188069409326171</v>
+        <v>-1.88069409326171E-3</v>
       </c>
       <c r="C21">
-        <v>5.1841760333083102e-05</v>
+        <v>5.1841760333083102E-5</v>
       </c>
       <c r="D21">
-        <v>-0.0103741431635685</v>
+        <v>-1.03741431635685E-2</v>
       </c>
       <c r="E21">
-        <v>5.7599050429216997e-05</v>
+        <v>5.7599050429216997E-5</v>
       </c>
       <c r="F21">
-        <v>-0.0192813651566941</v>
+        <v>-1.92813651566941E-2</v>
       </c>
       <c r="G21">
-        <v>9.6150731585761297e-05</v>
+        <v>9.6150731585761297E-5</v>
       </c>
       <c r="H21">
-        <v>-0.010833201879136899</v>
+        <v>-1.0833201879136899E-2</v>
       </c>
       <c r="I21">
-        <v>0.00013517001262568001</v>
+        <v>1.3517001262568001E-4</v>
       </c>
       <c r="J21">
-        <v>0.095000000000000001</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="K21">
-        <v>0.095000000000000001</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="L21">
-        <v>0.095000000000000001</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="M21">
-        <v>0.095000000000000001</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>9.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22">
-        <v>-0.00196222546133941</v>
+        <v>-1.96222546133941E-3</v>
       </c>
       <c r="C22">
-        <v>4.5900342267385702e-05</v>
+        <v>4.5900342267385702E-5</v>
       </c>
       <c r="D22">
-        <v>-0.010139638658091501</v>
+        <v>-1.0139638658091501E-2</v>
       </c>
       <c r="E22">
-        <v>6.3766210387500104e-05</v>
+        <v>6.3766210387500104E-5</v>
       </c>
       <c r="F22">
-        <v>-0.020127579603265899</v>
+        <v>-2.0127579603265899E-2</v>
       </c>
       <c r="G22">
-        <v>9.3094354325079802e-05</v>
+        <v>9.3094354325079802E-5</v>
       </c>
       <c r="H22">
-        <v>-0.0098627760060073805</v>
+        <v>-9.8627760060073805E-3</v>
       </c>
       <c r="I22">
-        <v>0.000101524242038476</v>
+        <v>1.01524242038476E-4</v>
       </c>
       <c r="J22">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="K22">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L22">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="M22">
-        <v>0.10000000000000001</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B23">
-        <v>-0.0020166569101412002</v>
+        <v>-2.0166569101412002E-3</v>
       </c>
       <c r="C23">
-        <v>4.64898917160376e-05</v>
+        <v>4.64898917160376E-5</v>
       </c>
       <c r="D23">
-        <v>-0.0100888961063444</v>
+        <v>-1.00888961063444E-2</v>
       </c>
       <c r="E23">
-        <v>9.2475219124284105e-05</v>
+        <v>9.2475219124284105E-5</v>
       </c>
       <c r="F23">
-        <v>-0.019784972994080399</v>
+        <v>-1.9784972994080399E-2</v>
       </c>
       <c r="G23">
-        <v>9.58208175138039e-05</v>
+        <v>9.58208175138039E-5</v>
       </c>
       <c r="H23">
-        <v>-0.0080869048639393201</v>
+        <v>-8.0869048639393201E-3</v>
       </c>
       <c r="I23">
-        <v>0.000121581839439923</v>
+        <v>1.21581839439923E-4</v>
       </c>
       <c r="J23">
         <v>0.105</v>
@@ -969,30 +1311,30 @@
         <v>0.105</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B24">
-        <v>-0.0020435308207603598</v>
+        <v>-2.0435308207603598E-3</v>
       </c>
       <c r="C24">
-        <v>4.6207732070384002e-05</v>
+        <v>4.6207732070384002E-5</v>
       </c>
       <c r="D24">
-        <v>-0.0125349830260364</v>
+        <v>-1.25349830260364E-2</v>
       </c>
       <c r="E24">
-        <v>0.00016119386648022501</v>
+        <v>1.6119386648022501E-4</v>
       </c>
       <c r="F24">
-        <v>-0.0203452229175447</v>
+        <v>-2.03452229175447E-2</v>
       </c>
       <c r="G24">
-        <v>9.0826657469727899e-05</v>
+        <v>9.0826657469727899E-5</v>
       </c>
       <c r="H24">
-        <v>-0.016974223398540399</v>
+        <v>-1.6974223398540399E-2</v>
       </c>
       <c r="I24">
-        <v>0.000123632387039249</v>
+        <v>1.23632387039249E-4</v>
       </c>
       <c r="J24">
         <v>0.11</v>
@@ -1007,30 +1349,30 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B25">
-        <v>-0.0022099612001010502</v>
+        <v>-2.2099612001010502E-3</v>
       </c>
       <c r="C25">
-        <v>4.9172361003870301e-05</v>
+        <v>4.9172361003870301E-5</v>
       </c>
       <c r="D25">
-        <v>-0.015921814132561898</v>
+        <v>-1.5921814132561898E-2</v>
       </c>
       <c r="E25">
-        <v>0.00011554251818205601</v>
+        <v>1.1554251818205601E-4</v>
       </c>
       <c r="F25">
-        <v>-0.0211286827119791</v>
+        <v>-2.11286827119791E-2</v>
       </c>
       <c r="G25">
-        <v>8.6498138457757206e-05</v>
+        <v>8.6498138457757206E-5</v>
       </c>
       <c r="H25">
-        <v>-0.0164998255595823</v>
+        <v>-1.64998255595823E-2</v>
       </c>
       <c r="I25">
-        <v>0.000121636642535473</v>
+        <v>1.21636642535473E-4</v>
       </c>
       <c r="J25">
         <v>0.115</v>
@@ -1045,30 +1387,30 @@
         <v>0.115</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26">
-        <v>-0.0022764899545988202</v>
+        <v>-2.2764899545988202E-3</v>
       </c>
       <c r="C26">
-        <v>4.7696895369437303e-05</v>
+        <v>4.7696895369437303E-5</v>
       </c>
       <c r="D26">
-        <v>-0.017145596941666501</v>
+        <v>-1.7145596941666501E-2</v>
       </c>
       <c r="E26">
-        <v>9.0766087487281801e-05</v>
+        <v>9.0766087487281801E-5</v>
       </c>
       <c r="F26">
-        <v>-0.0205612767029449</v>
+        <v>-2.05612767029449E-2</v>
       </c>
       <c r="G26">
-        <v>9.3035756465393099e-05</v>
+        <v>9.3035756465393099E-5</v>
       </c>
       <c r="H26">
-        <v>-0.018600671830249799</v>
+        <v>-1.8600671830249799E-2</v>
       </c>
       <c r="I26">
-        <v>0.000118236614387564</v>
+        <v>1.18236614387564E-4</v>
       </c>
       <c r="J26">
         <v>0.12</v>
@@ -1083,30 +1425,30 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27">
-        <v>-0.00235180414796856</v>
+        <v>-2.35180414796856E-3</v>
       </c>
       <c r="C27">
-        <v>4.69086499604721e-05</v>
+        <v>4.69086499604721E-5</v>
       </c>
       <c r="D27">
-        <v>-0.0164329006563095</v>
+        <v>-1.64329006563095E-2</v>
       </c>
       <c r="E27">
-        <v>8.8232792847954097e-05</v>
+        <v>8.8232792847954097E-5</v>
       </c>
       <c r="F27">
-        <v>-0.0199900758892671</v>
+        <v>-1.99900758892671E-2</v>
       </c>
       <c r="G27">
-        <v>8.0260110646389505e-05</v>
+        <v>8.0260110646389505E-5</v>
       </c>
       <c r="H27">
-        <v>-0.0197811967990471</v>
+        <v>-1.97811967990471E-2</v>
       </c>
       <c r="I27">
-        <v>0.00010171241607227</v>
+        <v>1.0171241607227E-4</v>
       </c>
       <c r="J27">
         <v>0.125</v>
@@ -1121,30 +1463,30 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B28">
-        <v>-0.0022996591252041599</v>
+        <v>-2.2996591252041599E-3</v>
       </c>
       <c r="C28">
-        <v>4.5519855748851598e-05</v>
+        <v>4.5519855748851598E-5</v>
       </c>
       <c r="D28">
-        <v>-0.0186912062763839</v>
+        <v>-1.86912062763839E-2</v>
       </c>
       <c r="E28">
-        <v>9.3692029928484994e-05</v>
+        <v>9.3692029928484994E-5</v>
       </c>
       <c r="F28">
-        <v>-0.019997504159046699</v>
+        <v>-1.9997504159046699E-2</v>
       </c>
       <c r="G28">
-        <v>6.9884895003098703e-05</v>
+        <v>6.9884895003098703E-5</v>
       </c>
       <c r="H28">
-        <v>-0.0190490579359259</v>
+        <v>-1.90490579359259E-2</v>
       </c>
       <c r="I28">
-        <v>9.0069115184854596e-05</v>
+        <v>9.0069115184854596E-5</v>
       </c>
       <c r="J28">
         <v>0.13</v>
@@ -1159,30 +1501,30 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B29">
-        <v>-0.00243741572101926</v>
+        <v>-2.43741572101926E-3</v>
       </c>
       <c r="C29">
-        <v>4.6627917260338999e-05</v>
+        <v>4.6627917260338999E-5</v>
       </c>
       <c r="D29">
-        <v>-0.018105547267353101</v>
+        <v>-1.8105547267353101E-2</v>
       </c>
       <c r="E29">
-        <v>0.00010178759156196699</v>
+        <v>1.0178759156196699E-4</v>
       </c>
       <c r="F29">
-        <v>-0.019824002577526301</v>
+        <v>-1.9824002577526301E-2</v>
       </c>
       <c r="G29">
-        <v>6.8478080977948906e-05</v>
+        <v>6.8478080977948906E-5</v>
       </c>
       <c r="H29">
-        <v>-0.0197269029726641</v>
+        <v>-1.97269029726641E-2</v>
       </c>
       <c r="I29">
-        <v>9.6338494641651001e-05</v>
+        <v>9.6338494641651001E-5</v>
       </c>
       <c r="J29">
         <v>0.13500000000000001</v>
@@ -1197,30 +1539,30 @@
         <v>0.13500000000000001</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B30">
-        <v>-0.0024324578462798299</v>
+        <v>-2.4324578462798299E-3</v>
       </c>
       <c r="C30">
-        <v>4.5882955249381697e-05</v>
+        <v>4.5882955249381697E-5</v>
       </c>
       <c r="D30">
-        <v>-0.019713610217695701</v>
+        <v>-1.9713610217695701E-2</v>
       </c>
       <c r="E30">
-        <v>7.9129569071999004e-05</v>
+        <v>7.9129569071999004E-5</v>
       </c>
       <c r="F30">
-        <v>-0.0198746131228754</v>
+        <v>-1.98746131228754E-2</v>
       </c>
       <c r="G30">
-        <v>8.5846658528960005e-05</v>
+        <v>8.5846658528960005E-5</v>
       </c>
       <c r="H30">
-        <v>-0.019955222228260398</v>
+        <v>-1.9955222228260398E-2</v>
       </c>
       <c r="I30">
-        <v>7.3584435696134396e-05</v>
+        <v>7.3584435696134396E-5</v>
       </c>
       <c r="J30">
         <v>0.14000000000000001</v>
@@ -1235,30 +1577,30 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B31">
-        <v>-0.0026149244541770699</v>
+        <v>-2.6149244541770699E-3</v>
       </c>
       <c r="C31">
-        <v>4.5536802076858502e-05</v>
+        <v>4.5536802076858502E-5</v>
       </c>
       <c r="D31">
-        <v>-0.0187223293911035</v>
+        <v>-1.87223293911035E-2</v>
       </c>
       <c r="E31">
-        <v>7.1532159322107094e-05</v>
+        <v>7.1532159322107094E-5</v>
       </c>
       <c r="F31">
-        <v>-0.019704537043997699</v>
+        <v>-1.9704537043997699E-2</v>
       </c>
       <c r="G31">
-        <v>7.1120938288083403e-05</v>
+        <v>7.1120938288083403E-5</v>
       </c>
       <c r="H31">
-        <v>-0.019468526697852401</v>
+        <v>-1.9468526697852401E-2</v>
       </c>
       <c r="I31">
-        <v>7.5369271222492303e-05</v>
+        <v>7.5369271222492303E-5</v>
       </c>
       <c r="J31">
         <v>0.14499999999999999</v>
@@ -1273,68 +1615,68 @@
         <v>0.14499999999999999</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B32">
-        <v>-0.0027281362734190399</v>
+        <v>-2.7281362734190399E-3</v>
       </c>
       <c r="C32">
-        <v>4.5802329322150401e-05</v>
+        <v>4.5802329322150401E-5</v>
       </c>
       <c r="D32">
-        <v>-0.019360216263016001</v>
+        <v>-1.9360216263016001E-2</v>
       </c>
       <c r="E32">
-        <v>7.4903697680105106e-05</v>
+        <v>7.4903697680105106E-5</v>
       </c>
       <c r="F32">
-        <v>-0.0199364560831903</v>
+        <v>-1.99364560831903E-2</v>
       </c>
       <c r="G32">
-        <v>7.8413679581698406e-05</v>
+        <v>7.8413679581698406E-5</v>
       </c>
       <c r="H32">
-        <v>-0.018575726402078999</v>
+        <v>-1.8575726402078999E-2</v>
       </c>
       <c r="I32">
-        <v>7.4469113702965102e-05</v>
+        <v>7.4469113702965102E-5</v>
       </c>
       <c r="J32">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="K32">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="L32">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="M32">
-        <v>0.14999999999999999</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33">
-        <v>-0.0027038456496019602</v>
+        <v>-2.7038456496019602E-3</v>
       </c>
       <c r="C33">
-        <v>4.6103275905078598e-05</v>
+        <v>4.6103275905078598E-5</v>
       </c>
       <c r="D33">
-        <v>-0.018474266445420901</v>
+        <v>-1.8474266445420901E-2</v>
       </c>
       <c r="E33">
-        <v>0.000116869734252979</v>
+        <v>1.16869734252979E-4</v>
       </c>
       <c r="F33">
-        <v>-0.0195002871955757</v>
+        <v>-1.95002871955757E-2</v>
       </c>
       <c r="G33">
-        <v>6.67892389801537e-05</v>
+        <v>6.67892389801537E-5</v>
       </c>
       <c r="H33">
-        <v>-0.018867758429019998</v>
+        <v>-1.8867758429019998E-2</v>
       </c>
       <c r="I33">
-        <v>6.9512866533152004e-05</v>
+        <v>6.9512866533152004E-5</v>
       </c>
       <c r="J33">
         <v>0.155</v>
@@ -1349,30 +1691,30 @@
         <v>0.155</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B34">
-        <v>-0.00280699306282134</v>
+        <v>-2.80699306282134E-3</v>
       </c>
       <c r="C34">
-        <v>4.57415468926148e-05</v>
+        <v>4.57415468926148E-5</v>
       </c>
       <c r="D34">
-        <v>-0.0189054864799077</v>
+        <v>-1.89054864799077E-2</v>
       </c>
       <c r="E34">
-        <v>6.5198938946966193e-05</v>
+        <v>6.5198938946966193E-5</v>
       </c>
       <c r="F34">
-        <v>-0.019718638632260799</v>
+        <v>-1.9718638632260799E-2</v>
       </c>
       <c r="G34">
-        <v>6.67712410296548e-05</v>
+        <v>6.67712410296548E-5</v>
       </c>
       <c r="H34">
-        <v>-0.018988169004320099</v>
+        <v>-1.8988169004320099E-2</v>
       </c>
       <c r="I34">
-        <v>6.3916148963857501e-05</v>
+        <v>6.3916148963857501E-5</v>
       </c>
       <c r="J34">
         <v>0.16</v>
@@ -1387,30 +1729,30 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35">
-        <v>-0.0028114512313985401</v>
+        <v>-2.8114512313985401E-3</v>
       </c>
       <c r="C35">
-        <v>4.62553545235389e-05</v>
+        <v>4.62553545235389E-5</v>
       </c>
       <c r="D35">
-        <v>-0.018567949073906902</v>
+        <v>-1.8567949073906902E-2</v>
       </c>
       <c r="E35">
-        <v>6.2037361769597002e-05</v>
+        <v>6.2037361769597002E-5</v>
       </c>
       <c r="F35">
-        <v>-0.019476424152094999</v>
+        <v>-1.9476424152094999E-2</v>
       </c>
       <c r="G35">
-        <v>8.0924149365410299e-05</v>
+        <v>8.0924149365410299E-5</v>
       </c>
       <c r="H35">
-        <v>-0.0182660656206916</v>
+        <v>-1.82660656206916E-2</v>
       </c>
       <c r="I35">
-        <v>6.1001369682051499e-05</v>
+        <v>6.1001369682051499E-5</v>
       </c>
       <c r="J35">
         <v>0.16500000000000001</v>
@@ -1425,68 +1767,68 @@
         <v>0.16500000000000001</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36">
-        <v>-0.0028741851266006401</v>
+        <v>-2.8741851266006401E-3</v>
       </c>
       <c r="C36">
-        <v>4.6498483976432303e-05</v>
+        <v>4.6498483976432303E-5</v>
       </c>
       <c r="D36">
-        <v>-0.017422389834580099</v>
+        <v>-1.7422389834580099E-2</v>
       </c>
       <c r="E36">
-        <v>0.000119020212009693</v>
+        <v>1.19020212009693E-4</v>
       </c>
       <c r="F36">
-        <v>-0.019438810987439801</v>
+        <v>-1.9438810987439801E-2</v>
       </c>
       <c r="G36">
-        <v>6.6159149649364503e-05</v>
+        <v>6.6159149649364503E-5</v>
       </c>
       <c r="H36">
-        <v>-0.017597102799565001</v>
+        <v>-1.7597102799565001E-2</v>
       </c>
       <c r="I36">
-        <v>7.4406524261133697e-05</v>
+        <v>7.4406524261133697E-5</v>
       </c>
       <c r="J36">
-        <v>0.17000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="K36">
-        <v>0.17000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="L36">
-        <v>0.17000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="M36">
-        <v>0.17000000000000001</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37">
-        <v>-0.0030658719996969701</v>
+        <v>-3.0658719996969701E-3</v>
       </c>
       <c r="C37">
-        <v>4.6756013697072601e-05</v>
+        <v>4.6756013697072601E-5</v>
       </c>
       <c r="D37">
-        <v>-0.017962815333094202</v>
+        <v>-1.7962815333094202E-2</v>
       </c>
       <c r="E37">
-        <v>5.7964621247771701e-05</v>
+        <v>5.7964621247771701E-5</v>
       </c>
       <c r="F37">
-        <v>-0.019527457166196999</v>
+        <v>-1.9527457166196999E-2</v>
       </c>
       <c r="G37">
-        <v>6.6603100174992798e-05</v>
+        <v>6.6603100174992798E-5</v>
       </c>
       <c r="H37">
-        <v>-0.0176696029547098</v>
+        <v>-1.76696029547098E-2</v>
       </c>
       <c r="I37">
-        <v>6.9342327557107795e-05</v>
+        <v>6.9342327557107795E-5</v>
       </c>
       <c r="J37">
         <v>0.17499999999999999</v>
@@ -1501,68 +1843,68 @@
         <v>0.17499999999999999</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B38">
-        <v>-0.0030648345733894199</v>
+        <v>-3.0648345733894199E-3</v>
       </c>
       <c r="C38">
-        <v>4.6859004763054602e-05</v>
+        <v>4.6859004763054602E-5</v>
       </c>
       <c r="D38">
-        <v>-0.018610075242397699</v>
+        <v>-1.8610075242397699E-2</v>
       </c>
       <c r="E38">
-        <v>9.1548633750095302e-05</v>
+        <v>9.1548633750095302E-5</v>
       </c>
       <c r="F38">
-        <v>-0.0196748273484567</v>
+        <v>-1.96748273484567E-2</v>
       </c>
       <c r="G38">
-        <v>6.9954003710809303e-05</v>
+        <v>6.9954003710809303E-5</v>
       </c>
       <c r="H38">
-        <v>-0.0187880072259279</v>
+        <v>-1.87880072259279E-2</v>
       </c>
       <c r="I38">
-        <v>6.4453760957897905e-05</v>
+        <v>6.4453760957897905E-5</v>
       </c>
       <c r="J38">
-        <v>0.17999999999999999</v>
+        <v>0.18</v>
       </c>
       <c r="K38">
-        <v>0.17999999999999999</v>
+        <v>0.18</v>
       </c>
       <c r="L38">
-        <v>0.17999999999999999</v>
+        <v>0.18</v>
       </c>
       <c r="M38">
-        <v>0.17999999999999999</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B39">
-        <v>-0.0032191390335258299</v>
+        <v>-3.2191390335258299E-3</v>
       </c>
       <c r="C39">
-        <v>4.6689100853879901e-05</v>
+        <v>4.6689100853879901E-5</v>
       </c>
       <c r="D39">
-        <v>-0.018554538365103901</v>
+        <v>-1.8554538365103901E-2</v>
       </c>
       <c r="E39">
-        <v>0.00010144375611649201</v>
+        <v>1.0144375611649201E-4</v>
       </c>
       <c r="F39">
-        <v>-0.019340032841076101</v>
+        <v>-1.9340032841076101E-2</v>
       </c>
       <c r="G39">
-        <v>7.8097663272109593e-05</v>
+        <v>7.8097663272109593E-5</v>
       </c>
       <c r="H39">
-        <v>-0.018595161602639399</v>
+        <v>-1.8595161602639399E-2</v>
       </c>
       <c r="I39">
-        <v>7.1483303717753197e-05</v>
+        <v>7.1483303717753197E-5</v>
       </c>
       <c r="J39">
         <v>0.185</v>
@@ -1577,30 +1919,30 @@
         <v>0.185</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B40">
-        <v>-0.0033478172592234599</v>
+        <v>-3.3478172592234599E-3</v>
       </c>
       <c r="C40">
-        <v>4.5757123563576203e-05</v>
+        <v>4.5757123563576203E-5</v>
       </c>
       <c r="D40">
-        <v>-0.018613311613192199</v>
+        <v>-1.8613311613192199E-2</v>
       </c>
       <c r="E40">
-        <v>8.9904363612627202e-05</v>
+        <v>8.9904363612627202E-5</v>
       </c>
       <c r="F40">
-        <v>-0.0195081958113991</v>
+        <v>-1.95081958113991E-2</v>
       </c>
       <c r="G40">
-        <v>6.63933956188115e-05</v>
+        <v>6.63933956188115E-5</v>
       </c>
       <c r="H40">
-        <v>-0.018430449897549599</v>
+        <v>-1.8430449897549599E-2</v>
       </c>
       <c r="I40">
-        <v>7.4036747997512596e-05</v>
+        <v>7.4036747997512596E-5</v>
       </c>
       <c r="J40">
         <v>0.19</v>
@@ -1615,30 +1957,30 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41">
-        <v>-0.0031937118163386301</v>
+        <v>-3.1937118163386301E-3</v>
       </c>
       <c r="C41">
-        <v>5.01507503154668e-05</v>
+        <v>5.01507503154668E-5</v>
       </c>
       <c r="D41">
-        <v>-0.018712669754000499</v>
+        <v>-1.8712669754000499E-2</v>
       </c>
       <c r="E41">
-        <v>8.0490196480605599e-05</v>
+        <v>8.0490196480605599E-5</v>
       </c>
       <c r="F41">
-        <v>-0.019520320033411399</v>
+        <v>-1.9520320033411399E-2</v>
       </c>
       <c r="G41">
-        <v>6.7564417564479906e-05</v>
+        <v>6.7564417564479906E-5</v>
       </c>
       <c r="H41">
-        <v>-0.017556330294930301</v>
+        <v>-1.7556330294930301E-2</v>
       </c>
       <c r="I41">
-        <v>0.00011770892817715</v>
+        <v>1.1770892817715E-4</v>
       </c>
       <c r="J41">
         <v>0.19500000000000001</v>
@@ -1653,68 +1995,68 @@
         <v>0.19500000000000001</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42">
-        <v>-0.0034969943144564598</v>
+        <v>-3.4969943144564598E-3</v>
       </c>
       <c r="C42">
-        <v>4.6230686125351599e-05</v>
+        <v>4.6230686125351599E-5</v>
       </c>
       <c r="D42">
-        <v>-0.018454878711534301</v>
+        <v>-1.8454878711534301E-2</v>
       </c>
       <c r="E42">
-        <v>6.7264551824597097e-05</v>
+        <v>6.7264551824597097E-5</v>
       </c>
       <c r="F42">
-        <v>-0.0195524629170944</v>
+        <v>-1.95524629170944E-2</v>
       </c>
       <c r="G42">
-        <v>6.8012292829048199e-05</v>
+        <v>6.8012292829048199E-5</v>
       </c>
       <c r="H42">
-        <v>-0.018091394205285799</v>
+        <v>-1.8091394205285799E-2</v>
       </c>
       <c r="I42">
-        <v>5.3696154486415199e-05</v>
+        <v>5.3696154486415199E-5</v>
       </c>
       <c r="J42">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="K42">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="L42">
-        <v>0.20000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="M42">
-        <v>0.20000000000000001</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43">
-        <v>-0.0035804591103513702</v>
+        <v>-3.5804591103513702E-3</v>
       </c>
       <c r="C43">
-        <v>4.6058068918333597e-05</v>
+        <v>4.6058068918333597E-5</v>
       </c>
       <c r="D43">
-        <v>-0.0177171500162903</v>
+        <v>-1.77171500162903E-2</v>
       </c>
       <c r="E43">
-        <v>0.000143584451531294</v>
+        <v>1.43584451531294E-4</v>
       </c>
       <c r="F43">
-        <v>-0.019428624095783598</v>
+        <v>-1.9428624095783598E-2</v>
       </c>
       <c r="G43">
-        <v>6.0398513152236598e-05</v>
+        <v>6.0398513152236598E-5</v>
       </c>
       <c r="H43">
-        <v>-0.017116181798428901</v>
+        <v>-1.7116181798428901E-2</v>
       </c>
       <c r="I43">
-        <v>0.000107087370322046</v>
+        <v>1.07087370322046E-4</v>
       </c>
       <c r="J43">
         <v>0.20499999999999999</v>
@@ -1729,68 +2071,68 @@
         <v>0.20499999999999999</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44">
-        <v>-0.00370975397571903</v>
+        <v>-3.70975397571903E-3</v>
       </c>
       <c r="C44">
-        <v>4.97091355724362e-05</v>
+        <v>4.97091355724362E-5</v>
       </c>
       <c r="D44">
-        <v>-0.0171525492275485</v>
+        <v>-1.71525492275485E-2</v>
       </c>
       <c r="E44">
-        <v>0.00018113638511502999</v>
+        <v>1.8113638511502999E-4</v>
       </c>
       <c r="F44">
-        <v>-0.019543918675823599</v>
+        <v>-1.9543918675823599E-2</v>
       </c>
       <c r="G44">
-        <v>6.4582111388965203e-05</v>
+        <v>6.4582111388965203E-5</v>
       </c>
       <c r="H44">
-        <v>-0.017078477663330701</v>
+        <v>-1.7078477663330701E-2</v>
       </c>
       <c r="I44">
-        <v>0.000118690382073201</v>
+        <v>1.18690382073201E-4</v>
       </c>
       <c r="J44">
-        <v>0.20999999999999999</v>
+        <v>0.21</v>
       </c>
       <c r="K44">
-        <v>0.20999999999999999</v>
+        <v>0.21</v>
       </c>
       <c r="L44">
-        <v>0.20999999999999999</v>
+        <v>0.21</v>
       </c>
       <c r="M44">
-        <v>0.20999999999999999</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45">
-        <v>-0.0037001153772679399</v>
+        <v>-3.7001153772679399E-3</v>
       </c>
       <c r="C45">
-        <v>4.6170069847581603e-05</v>
+        <v>4.6170069847581603E-5</v>
       </c>
       <c r="D45">
-        <v>-0.017687368562923501</v>
+        <v>-1.7687368562923501E-2</v>
       </c>
       <c r="E45">
-        <v>0.000160044029052438</v>
+        <v>1.60044029052438E-4</v>
       </c>
       <c r="F45">
-        <v>-0.019709112226717701</v>
+        <v>-1.9709112226717701E-2</v>
       </c>
       <c r="G45">
-        <v>6.0184179154877699e-05</v>
+        <v>6.0184179154877699E-5</v>
       </c>
       <c r="H45">
-        <v>-0.0168785673267846</v>
+        <v>-1.68785673267846E-2</v>
       </c>
       <c r="I45">
-        <v>0.000161260249214617</v>
+        <v>1.61260249214617E-4</v>
       </c>
       <c r="J45">
         <v>0.215</v>
@@ -1805,30 +2147,30 @@
         <v>0.215</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46">
-        <v>-0.0037692717038027902</v>
+        <v>-3.7692717038027902E-3</v>
       </c>
       <c r="C46">
-        <v>5.0931769464084101e-05</v>
+        <v>5.0931769464084101E-5</v>
       </c>
       <c r="D46">
-        <v>-0.017040112100870999</v>
+        <v>-1.7040112100870999E-2</v>
       </c>
       <c r="E46">
-        <v>0.000137972214179238</v>
+        <v>1.37972214179238E-4</v>
       </c>
       <c r="F46">
-        <v>-0.0196664236809393</v>
+        <v>-1.96664236809393E-2</v>
       </c>
       <c r="G46">
-        <v>6.1357277988993901e-05</v>
+        <v>6.1357277988993901E-5</v>
       </c>
       <c r="H46">
-        <v>-0.016958653480696299</v>
+        <v>-1.6958653480696299E-2</v>
       </c>
       <c r="I46">
-        <v>0.000118755020400947</v>
+        <v>1.18755020400947E-4</v>
       </c>
       <c r="J46">
         <v>0.22</v>
@@ -1843,30 +2185,30 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47">
-        <v>-0.0038632343718176701</v>
+        <v>-3.8632343718176701E-3</v>
       </c>
       <c r="C47">
-        <v>4.7797000402234503e-05</v>
+        <v>4.7797000402234503E-5</v>
       </c>
       <c r="D47">
-        <v>-0.017427597936276198</v>
+        <v>-1.7427597936276198E-2</v>
       </c>
       <c r="E47">
-        <v>0.00011405444973780801</v>
+        <v>1.1405444973780801E-4</v>
       </c>
       <c r="F47">
-        <v>-0.019604711589070501</v>
+        <v>-1.9604711589070501E-2</v>
       </c>
       <c r="G47">
-        <v>6.2033404007809094e-05</v>
+        <v>6.2033404007809094E-5</v>
       </c>
       <c r="H47">
-        <v>-0.016617223884562798</v>
+        <v>-1.6617223884562798E-2</v>
       </c>
       <c r="I47">
-        <v>0.000102479572908196</v>
+        <v>1.02479572908196E-4</v>
       </c>
       <c r="J47">
         <v>0.22500000000000001</v>
@@ -1881,68 +2223,68 @@
         <v>0.22500000000000001</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48">
-        <v>-0.0039705879571405797</v>
+        <v>-3.9705879571405797E-3</v>
       </c>
       <c r="C48">
-        <v>4.7927329300778198e-05</v>
+        <v>4.7927329300778198E-5</v>
       </c>
       <c r="D48">
-        <v>-0.017119339083637799</v>
+        <v>-1.7119339083637799E-2</v>
       </c>
       <c r="E48">
-        <v>0.00014733331146747801</v>
+        <v>1.4733331146747801E-4</v>
       </c>
       <c r="F48">
-        <v>-0.019309554572763399</v>
+        <v>-1.9309554572763399E-2</v>
       </c>
       <c r="G48">
-        <v>5.8794271712296698e-05</v>
+        <v>5.8794271712296698E-5</v>
       </c>
       <c r="H48">
-        <v>-0.016262240535972</v>
+        <v>-1.6262240535972E-2</v>
       </c>
       <c r="I48">
-        <v>0.00014675613779147501</v>
+        <v>1.4675613779147501E-4</v>
       </c>
       <c r="J48">
-        <v>0.23000000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="K48">
-        <v>0.23000000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="L48">
-        <v>0.23000000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="M48">
-        <v>0.23000000000000001</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49">
-        <v>-0.0041140081506318999</v>
+        <v>-4.1140081506318999E-3</v>
       </c>
       <c r="C49">
-        <v>4.9162251412693298e-05</v>
+        <v>4.9162251412693298E-5</v>
       </c>
       <c r="D49">
-        <v>-0.0170817329555789</v>
+        <v>-1.70817329555789E-2</v>
       </c>
       <c r="E49">
-        <v>0.000109977478525005</v>
+        <v>1.09977478525005E-4</v>
       </c>
       <c r="F49">
-        <v>-0.019476281086505402</v>
+        <v>-1.9476281086505402E-2</v>
       </c>
       <c r="G49">
-        <v>5.8224110983964298e-05</v>
+        <v>5.8224110983964298E-5</v>
       </c>
       <c r="H49">
-        <v>-0.016573031916449099</v>
+        <v>-1.6573031916449099E-2</v>
       </c>
       <c r="I49">
-        <v>0.00016464995132676701</v>
+        <v>1.6464995132676701E-4</v>
       </c>
       <c r="J49">
         <v>0.23499999999999999</v>
@@ -1957,144 +2299,144 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50">
-        <v>-0.00415889346847739</v>
+        <v>-4.15889346847739E-3</v>
       </c>
       <c r="C50">
-        <v>5.4636209887278202e-05</v>
+        <v>5.4636209887278202E-5</v>
       </c>
       <c r="D50">
-        <v>-0.0171250634665099</v>
+        <v>-1.71250634665099E-2</v>
       </c>
       <c r="E50">
-        <v>0.000138607029402968</v>
+        <v>1.38607029402968E-4</v>
       </c>
       <c r="F50">
-        <v>-0.019519570157337501</v>
+        <v>-1.9519570157337501E-2</v>
       </c>
       <c r="G50">
-        <v>7.0360148286179597e-05</v>
+        <v>7.0360148286179597E-5</v>
       </c>
       <c r="H50">
-        <v>-0.016788587895184101</v>
+        <v>-1.6788587895184101E-2</v>
       </c>
       <c r="I50">
-        <v>0.000139988158882576</v>
+        <v>1.39988158882576E-4</v>
       </c>
       <c r="J50">
-        <v>0.23999999999999999</v>
+        <v>0.24</v>
       </c>
       <c r="K50">
         <v>0.27500000000000002</v>
       </c>
       <c r="L50">
-        <v>0.23999999999999999</v>
+        <v>0.24</v>
       </c>
       <c r="M50">
         <v>0.27500000000000002</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51">
-        <v>-0.0044481085884705996</v>
+        <v>-4.4481085884705996E-3</v>
       </c>
       <c r="C51">
-        <v>4.86943850550312e-05</v>
+        <v>4.86943850550312E-5</v>
       </c>
       <c r="D51">
-        <v>-0.017021944156980402</v>
+        <v>-1.7021944156980402E-2</v>
       </c>
       <c r="E51">
-        <v>0.000167473263828954</v>
+        <v>1.67473263828954E-4</v>
       </c>
       <c r="F51">
-        <v>-0.019119047352325901</v>
+        <v>-1.9119047352325901E-2</v>
       </c>
       <c r="G51">
-        <v>5.8826307141244698e-05</v>
+        <v>5.8826307141244698E-5</v>
       </c>
       <c r="H51">
-        <v>-0.0173002535638371</v>
+        <v>-1.73002535638371E-2</v>
       </c>
       <c r="I51">
-        <v>0.000129999942456352</v>
+        <v>1.29999942456352E-4</v>
       </c>
       <c r="J51">
         <v>0.25</v>
       </c>
       <c r="K51">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="L51">
         <v>0.25</v>
       </c>
       <c r="M51">
-        <v>0.29999999999999999</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52">
-        <v>-0.0047949940690043104</v>
+        <v>-4.7949940690043104E-3</v>
       </c>
       <c r="C52">
-        <v>5.0457365714925101e-05</v>
+        <v>5.0457365714925101E-5</v>
       </c>
       <c r="D52">
-        <v>-0.016904507844311401</v>
+        <v>-1.6904507844311401E-2</v>
       </c>
       <c r="E52">
-        <v>5.5907377856930097e-05</v>
+        <v>5.5907377856930097E-5</v>
       </c>
       <c r="F52">
-        <v>-0.0194123802573117</v>
+        <v>-1.94123802573117E-2</v>
       </c>
       <c r="G52">
-        <v>7.06283503233115e-05</v>
+        <v>7.06283503233115E-5</v>
       </c>
       <c r="H52">
-        <v>-0.0175260451658572</v>
+        <v>-1.75260451658572E-2</v>
       </c>
       <c r="I52">
-        <v>8.0795225116137999e-05</v>
+        <v>8.0795225116137999E-5</v>
       </c>
       <c r="J52">
-        <v>0.27000000000000002</v>
+        <v>0.27</v>
       </c>
       <c r="K52">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="L52">
-        <v>0.27000000000000002</v>
+        <v>0.27</v>
       </c>
       <c r="M52">
         <v>0.32500000000000001</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53">
-        <v>-0.0053429704618533896</v>
+        <v>-5.3429704618533896E-3</v>
       </c>
       <c r="C53">
-        <v>5.3907579471029399e-05</v>
+        <v>5.3907579471029399E-5</v>
       </c>
       <c r="D53">
-        <v>-0.017014994634877299</v>
+        <v>-1.7014994634877299E-2</v>
       </c>
       <c r="E53">
-        <v>0.000100726261470812</v>
+        <v>1.00726261470812E-4</v>
       </c>
       <c r="F53">
-        <v>-0.019443861874081501</v>
+        <v>-1.9443861874081501E-2</v>
       </c>
       <c r="G53">
-        <v>5.90259286272291e-05</v>
+        <v>5.90259286272291E-5</v>
       </c>
       <c r="H53">
-        <v>-0.017641587313360199</v>
+        <v>-1.7641587313360199E-2</v>
       </c>
       <c r="I53">
-        <v>8.9462195466604997e-05</v>
+        <v>8.9462195466604997E-5</v>
       </c>
       <c r="J53">
         <v>0.28999999999999998</v>
@@ -2106,39 +2448,39 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="M53">
-        <v>0.34999999999999998</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54">
-        <v>-0.0060357562386256598</v>
+        <v>-6.0357562386256598E-3</v>
       </c>
       <c r="C54">
-        <v>4.8634516664269198e-05</v>
+        <v>4.8634516664269198E-5</v>
       </c>
       <c r="D54">
-        <v>-0.017181593842959</v>
+        <v>-1.7181593842959E-2</v>
       </c>
       <c r="E54">
-        <v>8.5986428275407502e-05</v>
+        <v>8.5986428275407502E-5</v>
       </c>
       <c r="F54">
-        <v>-0.019751985696597099</v>
+        <v>-1.9751985696597099E-2</v>
       </c>
       <c r="G54">
-        <v>8.5964615159980103e-05</v>
+        <v>8.5964615159980103E-5</v>
       </c>
       <c r="H54">
-        <v>-0.018053385579275601</v>
+        <v>-1.8053385579275601E-2</v>
       </c>
       <c r="I54">
-        <v>9.8452719158433405e-05</v>
+        <v>9.8452719158433405E-5</v>
       </c>
       <c r="J54">
         <v>0.31</v>
       </c>
       <c r="K54">
-        <v>0.32000000000000001</v>
+        <v>0.32</v>
       </c>
       <c r="L54">
         <v>0.31</v>
@@ -2147,534 +2489,535 @@
         <v>0.375</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55">
-        <v>-0.0065429500779967302</v>
+        <v>-6.5429500779967302E-3</v>
       </c>
       <c r="C55">
-        <v>5.8919950141146401e-05</v>
+        <v>5.8919950141146401E-5</v>
       </c>
       <c r="D55">
-        <v>-0.017080486711513399</v>
+        <v>-1.7080486711513399E-2</v>
       </c>
       <c r="E55">
-        <v>0.000116274561900966</v>
+        <v>1.16274561900966E-4</v>
       </c>
       <c r="F55">
-        <v>-0.019829503152237402</v>
+        <v>-1.9829503152237402E-2</v>
       </c>
       <c r="G55">
-        <v>7.0897337754565306e-05</v>
+        <v>7.0897337754565306E-5</v>
       </c>
       <c r="H55">
-        <v>-0.018403349671368599</v>
+        <v>-1.8403349671368599E-2</v>
       </c>
       <c r="I55">
-        <v>5.84955959950212e-05</v>
+        <v>5.84955959950212E-5</v>
       </c>
       <c r="J55">
-        <v>0.33000000000000002</v>
+        <v>0.33</v>
       </c>
       <c r="K55">
         <v>0.32500000000000001</v>
       </c>
       <c r="L55">
-        <v>0.33000000000000002</v>
+        <v>0.33</v>
       </c>
       <c r="M55">
-        <v>0.40000000000000002</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56">
-        <v>-0.0070697974153310396</v>
+        <v>-7.0697974153310396E-3</v>
       </c>
       <c r="C56">
-        <v>5.6773280369486898e-05</v>
+        <v>5.6773280369486898E-5</v>
       </c>
       <c r="D56">
-        <v>-0.017424310557213999</v>
+        <v>-1.7424310557213999E-2</v>
       </c>
       <c r="E56">
-        <v>8.7373021606489796e-05</v>
+        <v>8.7373021606489796E-5</v>
       </c>
       <c r="F56">
-        <v>-0.019690937810325101</v>
+        <v>-1.9690937810325101E-2</v>
       </c>
       <c r="G56">
-        <v>7.5049375970668897e-05</v>
+        <v>7.5049375970668897E-5</v>
       </c>
       <c r="H56">
-        <v>-0.019034407479598899</v>
+        <v>-1.9034407479598899E-2</v>
       </c>
       <c r="I56">
-        <v>7.1466955393763298e-05</v>
+        <v>7.1466955393763298E-5</v>
       </c>
       <c r="J56">
-        <v>0.34999999999999998</v>
+        <v>0.35</v>
       </c>
       <c r="K56">
-        <v>0.33000000000000002</v>
+        <v>0.33</v>
       </c>
       <c r="L56">
-        <v>0.34999999999999998</v>
+        <v>0.35</v>
       </c>
       <c r="M56">
         <v>0.42499999999999999</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57">
-        <v>-0.0077113300625709898</v>
+        <v>-7.7113300625709898E-3</v>
       </c>
       <c r="C57">
-        <v>5.5910542884646198e-05</v>
+        <v>5.5910542884646198E-5</v>
       </c>
       <c r="D57">
-        <v>-0.017388485478883099</v>
+        <v>-1.7388485478883099E-2</v>
       </c>
       <c r="E57">
-        <v>0.00012214821506416001</v>
+        <v>1.2214821506416001E-4</v>
       </c>
       <c r="F57">
-        <v>-0.020330432236953501</v>
+        <v>-2.0330432236953501E-2</v>
       </c>
       <c r="G57">
-        <v>5.5073991125556998e-05</v>
+        <v>5.5073991125556998E-5</v>
       </c>
       <c r="H57">
-        <v>-0.019193127601668001</v>
+        <v>-1.9193127601668001E-2</v>
       </c>
       <c r="I57">
-        <v>6.6875228805031697e-05</v>
+        <v>6.6875228805031697E-5</v>
       </c>
       <c r="J57">
         <v>0.37</v>
       </c>
       <c r="K57">
-        <v>0.34000000000000002</v>
+        <v>0.34</v>
       </c>
       <c r="L57">
         <v>0.37</v>
       </c>
       <c r="M57">
-        <v>0.45000000000000001</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58">
-        <v>-0.0085301849850590809</v>
+        <v>-8.5301849850590809E-3</v>
       </c>
       <c r="C58">
-        <v>5.6238630005634303e-05</v>
+        <v>5.6238630005634303E-5</v>
       </c>
       <c r="D58">
-        <v>-0.017544177798283701</v>
+        <v>-1.7544177798283701E-2</v>
       </c>
       <c r="E58">
-        <v>0.000113690950630098</v>
+        <v>1.13690950630098E-4</v>
       </c>
       <c r="F58">
-        <v>-0.020421321222946799</v>
+        <v>-2.0421321222946799E-2</v>
       </c>
       <c r="G58">
-        <v>9.1197246078953805e-05</v>
+        <v>9.1197246078953805E-5</v>
       </c>
       <c r="H58">
-        <v>-0.019747634302371801</v>
+        <v>-1.9747634302371801E-2</v>
       </c>
       <c r="I58">
-        <v>4.1992735271735303e-05</v>
+        <v>4.1992735271735303E-5</v>
       </c>
       <c r="J58">
-        <v>0.39000000000000001</v>
+        <v>0.39</v>
       </c>
       <c r="K58">
-        <v>0.34999999999999998</v>
+        <v>0.35</v>
       </c>
       <c r="L58">
-        <v>0.39000000000000001</v>
+        <v>0.39</v>
       </c>
       <c r="M58">
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59">
-        <v>-0.0092332129098019206</v>
+        <v>-9.2332129098019206E-3</v>
       </c>
       <c r="C59">
-        <v>5.1359363868596902e-05</v>
+        <v>5.1359363868596902E-5</v>
       </c>
       <c r="D59">
-        <v>-0.017047926459093601</v>
+        <v>-1.7047926459093601E-2</v>
       </c>
       <c r="E59">
-        <v>8.94179681567651e-05</v>
+        <v>8.94179681567651E-5</v>
       </c>
       <c r="F59">
-        <v>-0.020832303941595399</v>
+        <v>-2.0832303941595399E-2</v>
       </c>
       <c r="G59">
-        <v>8.0302464808343403e-05</v>
+        <v>8.0302464808343403E-5</v>
       </c>
       <c r="H59">
-        <v>-0.020185052283004101</v>
+        <v>-2.0185052283004101E-2</v>
       </c>
       <c r="I59">
-        <v>9.9226474720244602e-05</v>
+        <v>9.9226474720244602E-5</v>
       </c>
       <c r="J59">
-        <v>0.40999999999999998</v>
+        <v>0.41</v>
       </c>
       <c r="K59">
-        <v>0.34999999999999998</v>
+        <v>0.35</v>
       </c>
       <c r="L59">
-        <v>0.40999999999999998</v>
+        <v>0.41</v>
       </c>
       <c r="M59">
         <v>0.5</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60">
-        <v>-0.010009848083600999</v>
+        <v>-1.0009848083600999E-2</v>
       </c>
       <c r="C60">
-        <v>5.2180358816550099e-05</v>
+        <v>5.2180358816550099E-5</v>
       </c>
       <c r="D60">
-        <v>-0.017686812506464099</v>
+        <v>-1.7686812506464099E-2</v>
       </c>
       <c r="E60">
-        <v>0.000113142296094454</v>
+        <v>1.13142296094454E-4</v>
       </c>
       <c r="F60">
-        <v>-0.020915732153544999</v>
+        <v>-2.0915732153544999E-2</v>
       </c>
       <c r="G60">
-        <v>9.5605877992795604e-05</v>
+        <v>9.5605877992795604E-5</v>
       </c>
       <c r="H60">
-        <v>-0.020694053182825502</v>
+        <v>-2.0694053182825502E-2</v>
       </c>
       <c r="I60">
-        <v>4.7955169065771498e-05</v>
+        <v>4.7955169065771498E-5</v>
       </c>
       <c r="J60">
-        <v>0.42999999999999999</v>
+        <v>0.43</v>
       </c>
       <c r="K60">
-        <v>0.35999999999999999</v>
+        <v>0.36</v>
       </c>
       <c r="L60">
-        <v>0.42999999999999999</v>
+        <v>0.43</v>
       </c>
       <c r="M60">
         <v>0.52500000000000002</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61">
-        <v>-0.0109361158843611</v>
+        <v>-1.09361158843611E-2</v>
       </c>
       <c r="C61">
-        <v>5.2952026894535702e-05</v>
+        <v>5.2952026894535702E-5</v>
       </c>
       <c r="D61">
-        <v>-0.017830662095178099</v>
+        <v>-1.7830662095178099E-2</v>
       </c>
       <c r="E61">
-        <v>8.05523472130886e-05</v>
+        <v>8.05523472130886E-5</v>
       </c>
       <c r="F61">
-        <v>-0.021492708825641801</v>
+        <v>-2.1492708825641801E-2</v>
       </c>
       <c r="G61">
-        <v>9.1814811030204e-05</v>
+        <v>9.1814811030204E-5</v>
       </c>
       <c r="H61">
-        <v>-0.021056565741345099</v>
+        <v>-2.1056565741345099E-2</v>
       </c>
       <c r="I61">
-        <v>6.5111832348437306e-05</v>
+        <v>6.5111832348437306E-5</v>
       </c>
       <c r="J61">
-        <v>0.45000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="K61">
         <v>0.37</v>
       </c>
       <c r="L61">
-        <v>0.45000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="M61">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62">
-        <v>-0.0119953874387311</v>
+        <v>-1.19953874387311E-2</v>
       </c>
       <c r="C62">
-        <v>4.7632198177922099e-05</v>
+        <v>4.7632198177922099E-5</v>
       </c>
       <c r="D62">
-        <v>-0.017893218731125</v>
+        <v>-1.7893218731125E-2</v>
       </c>
       <c r="E62">
-        <v>0.000108008768491088</v>
+        <v>1.08008768491088E-4</v>
       </c>
       <c r="F62">
-        <v>-0.021818351099768499</v>
+        <v>-2.1818351099768499E-2</v>
       </c>
       <c r="G62">
-        <v>6.5121794503678995e-05</v>
+        <v>6.5121794503678995E-5</v>
       </c>
       <c r="H62">
-        <v>-0.021938660749525701</v>
+        <v>-2.1938660749525701E-2</v>
       </c>
       <c r="I62">
-        <v>5.4718653258345503e-05</v>
+        <v>5.4718653258345503E-5</v>
       </c>
       <c r="J62">
-        <v>0.46999999999999997</v>
+        <v>0.47</v>
       </c>
       <c r="K62">
         <v>0.375</v>
       </c>
       <c r="L62">
-        <v>0.46999999999999997</v>
+        <v>0.47</v>
       </c>
       <c r="M62">
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63">
-        <v>-0.0131426945265116</v>
+        <v>-1.31426945265116E-2</v>
       </c>
       <c r="C63">
-        <v>4.5965967596605999e-05</v>
+        <v>4.5965967596605999E-5</v>
       </c>
       <c r="D63">
-        <v>-0.017981509648707199</v>
+        <v>-1.7981509648707199E-2</v>
       </c>
       <c r="E63">
-        <v>8.4013974605812202e-05</v>
+        <v>8.4013974605812202E-5</v>
       </c>
       <c r="F63">
-        <v>-0.021960162448581701</v>
+        <v>-2.1960162448581701E-2</v>
       </c>
       <c r="G63">
-        <v>5.9901640026330797e-05</v>
+        <v>5.9901640026330797E-5</v>
       </c>
       <c r="H63">
-        <v>-0.0223042523216118</v>
+        <v>-2.23042523216118E-2</v>
       </c>
       <c r="I63">
-        <v>5.4787201029672098e-05</v>
+        <v>5.4787201029672098E-5</v>
       </c>
       <c r="J63">
-        <v>0.48999999999999999</v>
+        <v>0.49</v>
       </c>
       <c r="K63">
         <v>0.38</v>
       </c>
       <c r="L63">
-        <v>0.48999999999999999</v>
+        <v>0.49</v>
       </c>
       <c r="M63">
-        <v>0.59999999999999998</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64">
-        <v>-0.01434582046346</v>
+        <v>-1.434582046346E-2</v>
       </c>
       <c r="C64">
-        <v>4.6062397141803703e-05</v>
+        <v>4.6062397141803703E-5</v>
       </c>
       <c r="D64">
-        <v>-0.018196807081415901</v>
+        <v>-1.8196807081415901E-2</v>
       </c>
       <c r="E64">
-        <v>9.2293671620908104e-05</v>
+        <v>9.2293671620908104E-5</v>
       </c>
       <c r="F64">
-        <v>-0.022344891120151599</v>
+        <v>-2.2344891120151599E-2</v>
       </c>
       <c r="G64">
-        <v>0.000106942455739497</v>
+        <v>1.06942455739497E-4</v>
       </c>
       <c r="J64">
-        <v>0.51000000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="K64">
-        <v>0.39000000000000001</v>
-      </c>
-      <c r="L64">
-        <v>0.51000000000000001</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>0.39</v>
+      </c>
+      <c r="L64" s="1">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="65" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B65">
-        <v>-0.0155499657263596</v>
+        <v>-1.55499657263596E-2</v>
       </c>
       <c r="C65">
-        <v>4.6558005314226398e-05</v>
+        <v>4.6558005314226398E-5</v>
       </c>
       <c r="D65">
-        <v>-0.018266654723600801</v>
+        <v>-1.8266654723600801E-2</v>
       </c>
       <c r="E65">
-        <v>6.0060540071007797e-05</v>
+        <v>6.0060540071007797E-5</v>
       </c>
       <c r="F65">
-        <v>-0.022752952829917999</v>
+        <v>-2.2752952829917999E-2</v>
       </c>
       <c r="G65">
-        <v>8.7277414253632805e-05</v>
+        <v>8.7277414253632805E-5</v>
       </c>
       <c r="J65">
-        <v>0.53000000000000003</v>
+        <v>0.53</v>
       </c>
       <c r="K65">
-        <v>0.40000000000000002</v>
-      </c>
-      <c r="L65">
-        <v>0.53000000000000003</v>
-      </c>
-    </row>
-    <row r="66">
+        <v>0.4</v>
+      </c>
+      <c r="L65" s="1">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="66" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B66">
-        <v>-0.016827952530849202</v>
+        <v>-1.6827952530849202E-2</v>
       </c>
       <c r="C66">
-        <v>4.6138447942140701e-05</v>
+        <v>4.6138447942140701E-5</v>
       </c>
       <c r="D66">
-        <v>-0.018352752650174501</v>
+        <v>-1.8352752650174501E-2</v>
       </c>
       <c r="E66">
-        <v>0.000115682298808192</v>
+        <v>1.15682298808192E-4</v>
       </c>
       <c r="F66">
-        <v>-0.0230644991962962</v>
+        <v>-2.30644991962962E-2</v>
       </c>
       <c r="G66">
-        <v>0.00010491594476019</v>
+        <v>1.0491594476019E-4</v>
       </c>
       <c r="J66">
         <v>0.55000000000000004</v>
       </c>
       <c r="K66">
-        <v>0.40000000000000002</v>
-      </c>
-      <c r="L66">
+        <v>0.4</v>
+      </c>
+      <c r="L66" s="1">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D67">
-        <v>-0.018483921658770601</v>
+        <v>-1.8483921658770601E-2</v>
       </c>
       <c r="E67">
-        <v>5.0235702224316899e-05</v>
+        <v>5.0235702224316899E-5</v>
       </c>
       <c r="K67">
-        <v>0.40999999999999998</v>
-      </c>
-    </row>
-    <row r="68">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="68" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D68">
-        <v>-0.018841140870623801</v>
+        <v>-1.8841140870623801E-2</v>
       </c>
       <c r="E68">
-        <v>6.0539999341245197e-05</v>
+        <v>6.0539999341245197E-5</v>
       </c>
       <c r="K68">
         <v>0.42499999999999999</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D69">
-        <v>-0.0193060471369015</v>
+        <v>-1.93060471369015E-2</v>
       </c>
       <c r="E69">
-        <v>8.9157092850227399e-05</v>
+        <v>8.9157092850227399E-5</v>
       </c>
       <c r="K69">
-        <v>0.45000000000000001</v>
-      </c>
-    </row>
-    <row r="70">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="70" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D70">
-        <v>-0.019626797716521701</v>
+        <v>-1.9626797716521701E-2</v>
       </c>
       <c r="E70">
-        <v>8.3090379270030305e-05</v>
+        <v>8.3090379270030305E-5</v>
       </c>
       <c r="K70">
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D71">
-        <v>-0.019955786200856099</v>
+        <v>-1.9955786200856099E-2</v>
       </c>
       <c r="E71">
-        <v>0.000110024142664008</v>
+        <v>1.10024142664008E-4</v>
       </c>
       <c r="K71">
         <v>0.5</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D72">
-        <v>-0.0208336746162716</v>
+        <v>-2.08336746162716E-2</v>
       </c>
       <c r="E72">
-        <v>7.1862953943236494e-05</v>
+        <v>7.1862953943236494E-5</v>
       </c>
       <c r="K72">
         <v>0.52500000000000002</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D73">
-        <v>-0.020952382534600199</v>
+        <v>-2.0952382534600199E-2</v>
       </c>
       <c r="E73">
-        <v>7.2708391233658801e-05</v>
+        <v>7.2708391233658801E-5</v>
       </c>
       <c r="K73">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D74">
-        <v>-0.021114857814448801</v>
+        <v>-2.1114857814448801E-2</v>
       </c>
       <c r="E74">
-        <v>0.000102162971886211</v>
+        <v>1.02162971886211E-4</v>
       </c>
       <c r="K74">
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="2:12" x14ac:dyDescent="0.25">
       <c r="D75">
-        <v>-0.0221092271059933</v>
+        <v>-2.21092271059933E-2</v>
       </c>
       <c r="E75">
-        <v>6.3566076901895599e-05</v>
+        <v>6.3566076901895599E-5</v>
       </c>
       <c r="K75">
-        <v>0.59999999999999998</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>